<commit_message>
feat: implement TC-004 activity creation and publishing scenario
</commit_message>
<xml_diff>
--- a/populon-bqas-tymovy-excel.xlsx
+++ b/populon-bqas-tymovy-excel.xlsx
@@ -1703,17 +1703,17 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Vyhledání skupiny aktivním členem a ověření absence tlačítka Join group (prevence duplicity)</t>
+          <t>Založení a publikování nové aktivity ve skupině a kontrola jejího zobrazení na stránce Home</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>REQ-SOC-06 (Populon → Horní navigace → Search groups → Detail vyhledané skupiny)</t>
+          <t>REQ-ACT-01, REQ-ACT-02 (Populon → My groups → Administration → Activities → Add / Publish → Home)</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Ověřit pravidlo prevence duplicitního členství: pokud aktivní přihlášený člen vyhledá svou skupinu přes vyhledávač skupin (Search groups) a otevře její profil, systém rozpozná jeho existující členství a nenabízí tlačítko pro podání nové přihlášky (Join group), nýbrž nabízí správu stávajícího členství (Member information).</t>
+          <t>Ověřit, že administrátor skupiny může přes průvodce v administraci (Activities → Add) založit novou aktivitu s inkrementálním názvem Test (TK) [číslo], přiřadit jí pozvaného člena, aktivitu uložit (Save), publikovat přes nabídku Menu → Publish a následně na stránce Home ověřit, že se publikovaná aktivita pozvanému členovi zobrazila.</t>
         </is>
       </c>
       <c r="E5" s="18" t="inlineStr">
@@ -1723,38 +1723,47 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Člen (Tomáš Kanský) je přihlášen do Populonu a má aktivní členství ve skupině uu_2026_BQAS_team_1.</t>
+          <t>Uživatel (Tomáš Kanský) má aktivní členství a administrátorská práva ve skupině uu_2026_BQAS_team_1.</t>
         </is>
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>• Hledaná skupina: uu_2026_BQAS_team_1
-• Vyhledávací URL: /search</t>
+          <t>• Skupina: uu_2026_BQAS_team_1
+• Name (Název aktivity): Test (TK) [inkrementální číslo] (např. Test (TK) 2)
+• Pozvaný člen (Receivers): Tomáš Kanský</t>
         </is>
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
-          <t>1. Přihlásit se do systému jako aktivní člen skupiny.
-2. V horní navigační liště kliknout na Search groups (vyhledání skupin).
-3. Do vyhledávacího pole zadat název skupiny uu_2026_BQAS_team_1 a spustit vyhledávání.
-4. Ve výsledcích vyhledávání kliknout na odkaz skupiny uu_2026_BQAS_team_1.
-5. Na načtené stránce skupiny zkontrolovat sekci Basic info a provést pauzu pro ověření, že se nikde nenabízí tlačítko Join group, ale je k dispozici tlačítko Member information.
-6. Úspěšné dokončení testu a zavření prohlížeče.</t>
+          <t>1. Přihlásit se do systému Populon.
+2. V horní navigaci kliknout na My groups a vybrat skupinu uu_2026_BQAS_team_1.
+3. Na stránce skupiny kliknout na tlačítko Administration.
+4. V levém administračním menu otevřít sekci Activities a kliknout na tlačítko Add.
+5. Na 1. stránce průvodce (Basic info) vyplnit pole Name hodnotou Test (TK) [inkrementální číslo].
+6. Přejít přes Page 2 (Contact info) a Page 3 (Settings) na Page 4 (Receivers).
+7. V seznamu členů zaškrtnout člena, za kterého probíhá testování (Tomáš Kanský), a přejít na závěrečnou stránku průvodce (Summary).
+8. Kliknout na tlačítko Save pro uložení aktivity.
+9. V přehledu aktivit u nově vytvořené položky rozbalit tlačítko Menu a zvolit Publish.
+10. V horní navigaci přejít na stránku Home a zkontrolovat, zda se nově publikovaná aktivita zobrazila v přehledu.</t>
         </is>
       </c>
       <c r="I5" s="18" t="inlineStr">
         <is>
-          <t>1. Uživatel je úspěšně přihlášen na Dashboard.
-2. Otevře se stránka vyhledávače skupin /search.
-3. Systém vyhledá požadovanou skupinu a zobrazí ji v tabulce výsledků.
-4. Zobrazí se veřejný profil skupiny uu_2026_BQAS_team_1.
-5. Systém aktivnímu členovi nenabízí podání duplicitní přihlášky (tlačítko Join group chybí) a zobrazuje tlačítko Member information pro správu existujícího členství.
-6. Test je úspěšně dokončen a prohlížeč se korektně zavře.</t>
+          <t>1. Uživatel je úspěšně přihlášen.
+2. Zobrazí se profil skupiny uu_2026_BQAS_team_1.
+3. Otevře se administrační rozhraní skupiny (/manage/dashboard).
+4. Otevře se průvodce vytvořením nové aktivity na kroku 1 Basic info.
+5. Pole Name přijme zadaný název Test (TK) [inkrementální číslo].
+6. Průvodce plynule přejde přes Page 2 a Page 3 na krok 4 Receivers.
+7. Člen Tomáš Kanský je zaškrtnut a na souhrnné stránce (Summary) je uveden počet pozvaných členů (Invited members: 1).
+8. Aktivita se uloží do tabulky aktivit ve stavu UNPUBLISHED.
+9. Po akci Menu → Publish se stav aktivity v tabulce změní na PUBLISHED.
+10. Na stránce Home (/usercard) je nově publikovaná aktivita Test (TK) [inkrementální číslo] viditelně zobrazena v přehledu aktivit.</t>
         </is>
       </c>
       <c r="J5" s="18" t="inlineStr">
         <is>
-          <t>Skutečný výsledek plně odpovídá očekávanému chování. Vyhledání i prokliknutí proběhnou korektně a systém přihlášenému členovi tlačítko Join group nezobrazí, čímž spolehlivě brání duplicitě.</t>
+          <t>Skutečný výsledek plně odpovídá očekávanému. Aktivita byla přes průvodce úspěšně založena, uložena, publikována přes Menu → Publish a ihned se zobrazila na stránce Home.</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -1764,7 +1773,7 @@
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>Scénář je plně automatizován v Playwright testu TC-004 (TK) v tests/scenarios.spec.ts.</t>
+          <t>Scénář je plně automatizován v Playwright testu TC-004 (TK) v tests/scenarios.spec.ts (automaticky inkrementuje číslo aktivity Test (TK) N).</t>
         </is>
       </c>
     </row>

</xml_diff>